<commit_message>
Regenerate the annotation workbook against the current chunking
build_annotation_sheet.py now reads the snapshot store rather than a flat
file, so the judgement grid matches the chunking actually in use.
</commit_message>
<xml_diff>
--- a/results/annotation_sheet.xlsx
+++ b/results/annotation_sheet.xlsx
@@ -937,17 +937,17 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>A Subclass 500 student visa holder in Australia can generally work part-time during their studies, with the following restrictions:  - Up to 20 hours per week while classes are in session. - Unlimited hours during school holidays.  It's important to note that these conditions may vary depending on the specific terms of your visa and the requirements set by the Australian Government. Always refer to the official Department of Home Affairs website or consult with a migration agent for the most accurate and up-to-date information related to your individual circumstances.</t>
+          <t>A Subclass 500 student visa holder in Australia can generally work part-time during their studies, with the following restrictions:  - Up to 20 hours per week while classes are in session. - Unlimited hours during school holidays.  It's important to note that these conditions may vary depending on the specific terms of your visa and the requirements set by the Department of Home Affairs. Always refer to the official Australian Government guidelines or consult with a migration agent or your visa sponsor for accurate, up-to-date information.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>A Subclass 500 Student visa holder can work up to 48 hours per fortnight while their course is in session. [Source: subclass_500_student.txt]</t>
+          <t>A Subclass 500 student visa holder can work up to 48 hours a fortnight while their course of study or training is in session. [Source: subclass_500_student.txt]</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>subclass_417_working_holiday.txt (0.827); subclass_485_temporary_graduate.txt (0.815); subclass_482_skills_in_demand.txt (0.781)</t>
+          <t>subclass_500_student.txt (0.829); subclass_485_temporary_graduate.txt (0.812); subclass_500_student.txt (0.786)</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr"/>
@@ -986,17 +986,17 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>The maximum stay for a Subclass 485 Temporary Graduate (Post-Study Work) visa is generally up to 3 years, but this can vary based on your study history. Here are some key points:  1. **First Degree**: For the first degree completed in Australia, you can stay for up to 2 years.  2. **Subsequent Degrees**:     - If it's a higher degree by research (PhD or equivalent), you can stay for up to 4 years.    - For other subsequent degrees, you can stay for up to 3 years.  It's important to note that these periods are cumulative and do not reset with each new visa application. Additionally, the Department of Home Affairs may consider factors such as your employment history and compliance with the conditions of previous visas when determining eligibility.  Always check the latest official guidelines from the Australian Government or consult with an immigration advisor for the most accurate and up-to-date information.</t>
+          <t>The maximum stay for a Subclass 485 Temporary Graduate (Post-Study Work) visa is generally up to 3 years, but this can be extended to up to 4 years under certain conditions.   Here are some key points:  1. **Initial Visa**: The initial visa allows a stay of up to 2 years. 2. **Eligibility for Extension**: If you meet specific criteria (such as having worked in an eligible occupation, or being employed by a recognized employer), you may be eligible for an extension that brings the total stay to up to 4 years.  To qualify for the full 4-year period, you typically need to: - Have been employed in an eligible occupation for at least 12 months after your graduation. - Be employed by a recognized employer (such as a business with a turnover of over $2 million).  It's important to check the latest Department of Home Affairs guidelines and policies, as these can change.</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>The maximum stay on a Subclass 485 Temporary Graduate visa in the Post-Higher Education Work stream can be up to four years. This information is specific to the conditions of the Post-Higher Education Work stream and should be verified with the individual's visa grant notice or VEVO for precise details.</t>
+          <t>The maximum stay on a Subclass 485 Temporary Graduate visa in the Post-Higher Education Work stream is between 1 and 2 years, depending on the regional location of the graduating institution and the regional area lived in while holding the visa. Source: subclass_485_temporary_graduate.txt</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>subclass_485_temporary_graduate.txt (0.804); subclass_482_skills_in_demand.txt (0.795); subclass_485_temporary_graduate.txt (0.789)</t>
+          <t>subclass_485_temporary_graduate.txt (0.868); subclass_485_temporary_graduate.txt (0.844); subclass_485_temporary_graduate.txt (0.837)</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
@@ -1035,17 +1035,17 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Yes, a Subclass 482 Skills in Demand visa does require employer sponsorship. This visa is designed to address skill shortages in specific occupations and industries in Australia. To apply for this visa, you must have an approved job offer from an Australian employer who has demonstrated that they cannot find an Australian worker to fill the position.  The employer will need to provide evidence of their efforts to recruit locally before offering the position to a skilled migrant. They must also show that employing a foreign worker is necessary and that the employment will not negatively impact the wages or conditions of existing Australian workers.  It's important to note that while the visa itself requires sponsorship, there are different types of Subclass 482 visas (e.g., temporary and permanent), which may have varying requirements. Always consult the latest information from the Department of Home Affairs or seek professional advice to ensure you meet all the necessary criteria for your specific situation.</t>
+          <t>Yes, a Subclass 482 Skills in Demand visa does require employer sponsorship. This visa is designed to address skill shortages in specific industries and occupations within Australia. To apply for this visa, you must have an approved job offer from an Australian employer who has demonstrated that they cannot find an appropriately skilled local worker.  The process involves several steps:  1. The Australian employer must first obtain a nomination from a state or territory government. 2. Once nominated, the employer can then submit a Subclass 482 application on your behalf. 3. If approved, you will be granted temporary work rights in Australia to perform the job offered.  It's important to note that while this visa allows for longer-term stays compared to other temporary work visas (up to four years and six months), it is still a temporary visa, meaning it does not lead directly to permanent residency unless additional steps are taken.</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Yes, a Subclass 482 Skills in Demand visa requires employer sponsorship. This is an employer-sponsored temporary visa designed to fill positions that cannot be filled by suitably skilled Australian workers.</t>
+          <t>Yes, a Subclass 482 Skills in Demand visa requires employer sponsorship. This is an employer-sponsored temporary visa. [Source: subclass_482_skills_in_demand.txt]</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>subclass_482_skills_in_demand.txt (0.852); subclass_482_skills_in_demand.txt (0.817); whm_6_month_work_limitation.txt (0.725)</t>
+          <t>subclass_482_skills_in_demand.txt (0.886); subclass_482_skills_in_demand.txt (0.843); subclass_482_skills_in_demand.txt (0.813)</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
@@ -1084,17 +1084,17 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>A Subclass 417 Working Holiday visa holder is generally not permitted to work for the same employer for more than six months, regardless of the industry. This restriction applies across all sectors, including tourism and hospitality.  However, there are some important points to consider:  1. **Continuous Employment**: The six-month period starts from the first day you begin working for a particular employer. If you leave that job and return to work for them later, it would be considered continuous employment, and the six-month limit still applies.  2. **Change of Employer**: You can change employers after your initial six months with one employer, but you must ensure you are not extending your stay beyond the permitted 12 months in total under this visa type.  3. **Other Employment**: If you work for a different employer within the same organization (e.g., moving from one branch to another), it may be considered continuous employment and could count towards the six-month limit.  4. **Visa Conditions**: Always check your specific visa conditions, as there might be variations depending on when your visa was granted or any changes in immigration policies.  5. **Employment Contracts**: Ensure that any employment contract complies with these restrictions to avoid potential issues with your visa status.  If you have concerns about working for the same employer for more than six months, it's advisable to consult with an immigration lawyer or the Department of Home Affairs directly for specific guidance tailored to your situation.</t>
+          <t>A Subclass 417 Working Holiday visa holder is generally not permitted to work for the same employer for more than six months, regardless of the industry. This restriction applies across all sectors, including tourism and hospitality.  However, there are some important points to consider:  1. **Employer Change**: If you leave one employer after working for them for up to 6 months, you can then take up employment with a different organization within the same six-month period without violating your visa conditions.  2. **Continuous Employment**: The six-month limit is based on continuous employment. If you have breaks in employment (e.g., taking time off or changing employers), this does not reset the clock for the six-month period.  3. **Industry-Specific Restrictions**: While there are no specific industry restrictions, it's important to note that working in a tourism and hospitality role might be more challenging due to seasonal variations and potential changes in employer needs.  4. **Visa Conditions**: Always refer to your specific visa conditions or consult with an immigration officer for precise guidance, as policies can change.  In summary, while you are allowed to work for the same employer for up to six months, you cannot extend this period by working continuously without changing employers.</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>No, a Subclass 417 Working Holiday visa holder cannot work for the same employer for more than 6 months. This is due to the specific 6-month work limitation with the same employer (condition 8547) that applies to subclass 417 visas as stated in the [subclass_417_working_holiday.txt] document.</t>
+          <t>For Subclass 417 Working Holiday visa holders, there is a specific work limitation that applies. According to the subclass 417 rules, holders must complete 6 months of specified subclass 417 work but are generally required to rotate employer or location every 6 months due to visa condition 8547 — unless an exemption applies.  Therefore, a Subclass 417 Working Holiday visa holder cannot work for the same employer for more than 6 months without potentially breaching their visa conditions. This restriction is in place regardless of the sector (such as tourism and hospitality) they are working in.  For specific exemptions or further details on this condition, please refer to the WHM 6 month work limitation document or contact a registered migration agent or the Department of Home Affairs directly.</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>subclass_417_working_holiday.txt (0.839); whm_6_month_work_limitation.txt (0.823); subclass_417_working_holiday.txt (0.803)</t>
+          <t>subclass_417_working_holiday.txt (0.855); subclass_417_working_holiday.txt (0.842); subclass_417_working_holiday.txt (0.832)</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -1133,17 +1133,17 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>I'm sorry, but there doesn't appear to be any widely recognized or official immigration condition known as "condition 8547." It's possible that this might be a specific reference within a certain context or jurisdiction, such as Australia (which uses the term "conditions" for visa requirements), but I couldn't find any standardized information about it.  In Australian migration law, there are various conditions that can apply to different types of visas. For example:  1. **8503 Temporary Activity Zone Condition**: This condition applies to holders of certain temporary activity zone visas and requires them to remain within the designated area while in Australia.  2. **8546 Character Requirement**: This is a condition that may be imposed on some visa subclasses, requiring the applicant to have no criminal convictions or other character issues that would make them unsuitable for entry into Australia.  If you're referring to a specific program or context, could you provide more details? That way, I can give you a more accurate answer.</t>
+          <t>I'm sorry, but there doesn't appear to be any widely recognized or official immigration condition known as "condition 8547." It's possible this could be a specific reference within a certain context or jurisdiction that I don't have information about.  In general, when discussing visa conditions:  - Different countries and regions have their own unique sets of rules and regulations for various types of visas. - These conditions can vary widely depending on the type of visa (e.g., student, work, tourist) and the country's immigration policies. - Conditions might include requirements like maintaining health insurance, not engaging in unauthorized employment, or leaving the country by a certain date.  If you could provide more context about where you heard this reference to "condition 8547" or which country's visa system it might be related to, I would be better able to assist you with accurate information.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Condition 8547 applies to anyone in Australia who holds a Working Holiday Maker (WHM) visa, specifically Subclass 417 (Working Holiday) and Subclass 462 (Work and Holiday) visas. It also applies to individuals holding a Bridging visa with condition 8547 imposed. This condition restricts work to no more than six months with the same employer unless an exemption applies or written approval has been obtained.  This information is sourced from [whm_6_month_work_limitation.txt] and [subclass_417_working_holiday.txt].</t>
+          <t>Condition 8547 applies to anyone in Australia who holds a Working Holiday Maker (WHM) visa, specifically Subclass 417 (Working Holiday) and Subclass 462 (Work and Holiday) visas. It also applies to individuals holding a Bridging visa with condition 8547 imposed. This condition is detailed in the document "whm_6_month_work_limitation.txt".</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>whm_6_month_work_limitation.txt (0.81); subclass_417_working_holiday.txt (0.701); whm_6_month_work_limitation.txt (0.698)</t>
+          <t>whm_6_month_work_limitation.txt (0.783); whm_6_month_work_limitation.txt (0.718); whm_6_month_work_limitation.txt (0.705)</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr"/>
@@ -1182,17 +1182,17 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>The cost of a Subclass 500 Student Visa in Australia can vary depending on several factors, including your country of citizenship and the type of course you are undertaking. As of my last update, here is a general overview:  1. **Citizenship/Residency Status**:     - Citizens or permanent residents of Australia: Free    - Other citizens: There is no separate student visa fee for these applicants.  2. **Course Duration and Type**:    - The cost can vary based on the length and type of course you are enrolled in.    - For example, a short-term study (up to 3 months) might have different costs compared to a full-time degree program.  3. **Application Fees**:     - There is no application fee for student visas as of recent changes by the Australian government.  4. **Health Insurance and Other Costs**:    - You will need to arrange private health insurance, which can cost around AUD $1,000 per year.    - Accommodation, living expenses, textbooks, and other course-related costs are additional and vary widely based on your personal circumstances and location in Australia.  For the most accurate and up-to-date information, it's recommended to check the official Australian Government Department of Home Affairs website or contact an authorized migration agent.</t>
+          <t>The cost of a Subclass 500 Student Visa in Australia can vary depending on several factors, including your country of citizenship, the type of course you're enrolled in, and whether it's full-time or part-time study. As of my last update, here are some general costs:  1. **Citizenship**:     - Full-time students from certain countries (e.g., India, Pakistan) pay a lower fee than others.     2. **Non-citizen students**:    - The cost can range significantly based on your country of citizenship and the type of course.  3. **Course Type**:    - Full-time courses generally have higher fees compared to part-time courses.  4. **Additional Fees**:    - There are also additional fees for things like medical clearance, student health insurance, and other government charges that may apply.  For the most accurate and up-to-date information, you should visit the official Australian Government Department of Home Affairs website or contact their customer service directly. They provide detailed fee schedules based on your specific circumstances.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>The cost of a Subclass 500 Student visa is from AUD2,500.00. Concessions apply in limited circumstances. This information can be found in the document titled "Subclass 500 Student visa — Overview".</t>
+          <t>The cost for a Subclass 500 Student visa is AUD2,500.00, with lower costs applying to eligible Pacific Island and Timor-Leste citizens, eligible ASEAN citizens, and applicants in the ELICOS and Non-Award sector who lodge a valid Student visa application. Source: [subclass_500_student.txt]</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>subclass_500_student.txt (0.777); subclass_500_student.txt (0.724); subclass_482_skills_in_demand.txt (0.701)</t>
+          <t>subclass_500_student.txt (0.843); subclass_500_student.txt (0.808); subclass_500_student.txt (0.751)</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
@@ -1231,17 +1231,17 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>The number of hours you're allowed to work per fortnight on your visa depends on the specific type of visa you hold and any conditions associated with it. Here are some general guidelines:  1. **Student Visa (Subclass 500)**: You can usually work up to 40 hours a fortnight during term time, but this may vary depending on your course level.  2. **Working Holiday Visa (Subclass 417 or 462)**: You are generally allowed to work full-time (usually defined as 38-40 hours per week) for the duration of your visa.  3. **Temporary Skill Shortage Visa (Subclass 482)**: The number of hours you can work depends on the occupation and employer, but it typically allows for full-time employment.  4. **Other Visas**: For other types of visas, check the specific conditions attached to your visa or consult the Department of Home Affairs website for detailed information.  It's important to review the specific terms and conditions of your visa, as these can vary widely depending on the type of visa you hold. If you're unsure about your work rights, it's best to contact the Department of Home Affairs or a registered migration agent for accurate advice.</t>
+          <t>The number of hours you're allowed to work per fortnight on your visa depends on the specific type of visa you hold and any conditions associated with it. Here are some general guidelines:  1. **Student Visa (Subclass 500)**: Typically, students can work up to 20 hours per week during term time and unlimited hours during school holidays.  2. **Working Holiday Visa (Subclass 417 or 462)**: Holders of this visa are generally allowed to work full-time (usually defined as 38 hours per week) but must be actively seeking employment for at least two weeks before they can start working.  3. **Temporary Work Visa (Subclass 457, 482, or 485)**: The number of hours you're allowed to work can vary depending on the specific visa subclass and any conditions attached by the Department of Home Affairs.  4. **Other Visas**: For other types of visas, such as business or employment-related visas (e.g., Subclass 186, 187, 132), you should check the specific visa requirements and conditions provided by the Australian Government.  To get accurate information about your specific visa type and work rights, it's best to consult the official Australian Government Department of Home Affairs website or contact their customer service directly. They can provide detailed guidance based on your individual circumstances.</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>The answer varies depending on your visa subclass:  - For Subclass 417 holders, there is no stated fortnightly work-hour cap; they can work unlimited hours but must generally rotate employer/location every 6 months. (subclass_417_working_holiday.txt) - For Subclass 500 Student visa holders, the cap is 48 hours per fortnight while their course is in session. (subclass_417_working_holiday.txt) - For Subclass 485 Temporary Graduate visa holders, there is no stated fortnightly work-hour cap; they can work in Australia under their stream conditions as specified in their visa grant notice/VEVO. (subclass_485_temporary_graduate.txt)  I don't have enough information in my sources to answer that.</t>
+          <t>That's a case-specific question — please contact a registered migration agent or the Department of Home Affairs directly. The subclass 417 Working Holiday visa does not have a stated fortnightly work-hour cap, but holders are subject to condition 8547 which limits working for the same employer to a maximum of 6 months. For more specific details about your individual circumstances and any conditions attached to your visa grant, you should check your visa grant notice/VEVO or contact the relevant authorities directly.</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>subclass_417_working_holiday.txt (0.762); whm_6_month_work_limitation.txt (0.752); subclass_485_temporary_graduate.txt (0.75)</t>
+          <t>subclass_417_working_holiday.txt (0.743); whm_6_month_work_limitation.txt (0.734); subclass_485_temporary_graduate.txt (0.731)</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr"/>
@@ -1280,17 +1280,17 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>The duration of your employment with an employer is generally not limited to six months by default; it depends on the specific terms outlined in your employment contract or agreement, local labor laws, and company policies.  Here are some key points to consider:  1. **Employment Contract**: Check if there's a clause specifying the term of your employment. Some contracts may have fixed-term agreements that last for more than six months.  2. **Local Labor Laws**: Different countries have different regulations regarding employment duration. For example, in many places, there are no legal restrictions on how long you can work for one employer, but some might have specific rules about renewals or terminations after a certain period.  3. **Company Policies**: Some companies may have internal policies that limit the length of continuous service for various reasons (e.g., to promote employee mobility). However, this is less common and usually not a legal requirement.  4. **Renewal Options**: If you're working under a contract with a fixed term, it can often be renewed upon mutual agreement between you and your employer.  5. **Performance Reviews**: Regular performance reviews can help ensure that both parties are satisfied with the arrangement, which might lead to continued employment beyond six months.  If you have concerns about the duration of your employment or any specific terms in your contract, it's a good idea to discuss these directly with your employer or seek advice from an HR representative.</t>
+          <t>The duration of your employment with an employer is generally not limited to six months by law, unless there's a specific contract or agreement that stipulates such a term. Most employment relationships are open-ended and can continue as long as both parties agree.  However, there might be some exceptions depending on the context:  1. **Internships**: Many internships have a defined duration, often around 3 to 6 months. 2. **Fixed-term contracts**: Some contracts may specify a fixed term of employment (e.g., for a project or specific period), after which the contract ends unless renewed. 3. **Seasonal work**: In some industries, like agriculture or tourism, seasonal work might be structured with defined periods.  If you have any concerns about your employment duration, it's best to review your employment agreement or speak with HR. If there are no explicit terms limiting your tenure, you can typically continue working for the same employer as long as both parties agree and comply with local labor laws.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>The ability to work for the same employer for more than 6 months depends on several factors. If your work does not fall under any of the specified exemptions (different locations, plant and animal cultivation, natural disaster recovery, critical sectors, or certain industries in Northern Australia), you can only work for the same employer for a maximum of 6 months while holding a WHM visa.  If you need to work longer than 6 months, you may be given permission under specific conditions: - You have applied for a visa allowing ongoing full-time work and are awaiting the outcome. - The work is critical to your employer, with a supporting letter attached to the request.  You can apply via the online form "Permission to work longer than 6 months." Continue working while awaiting a written decision if you submit the request before the 6-month period ends. If submitted after the 6 months ended, you must stop working for that employer until a decision is made.  For more detailed information on exemptions and specific scenarios, refer to the source document "whm_6_month_work_limitation.txt."</t>
+          <t>Yes, you can work for the same employer for more than 6 months if your work falls under one of the specified exemptions. These include working in different locations for the same employer, plant and animal cultivation anywhere in Australia, natural disaster recovery work anywhere in Australia, critical sectors anywhere in Australia (such as agriculture, health, aged and disability care, childcare, tourism and hospitality), or certain industries in Northern Australia only (fishing and pearling, tree farming and felling, construction, mining).  For more specific details on these exemptions, refer to the source document "Condition 8547 — WHM 6 month work limitation (Subclass 417 and 462)".</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>whm_6_month_work_limitation.txt (0.793); whm_6_month_work_limitation.txt (0.769); whm_6_month_work_limitation.txt (0.763)</t>
+          <t>whm_6_month_work_limitation.txt (0.822); whm_6_month_work_limitation.txt (0.786); whm_6_month_work_limitation.txt (0.765)</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
@@ -1329,17 +1329,17 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Congratulations on graduating! The specifics of your post-graduation visa (PGV) will depend on the type of visa you have been granted. Here’s a general overview based on common scenarios:  ### Post-Study Work Visa (PSW) If you are eligible for a PSW, which is typically granted to international students who have completed their studies in Australia, here's what you can expect:  1. **Duration:**    - For most bachelor's degrees, the initial PSW visa allows you to stay in Australia for up to 2 years.    - If your degree was part of a combined program (e.g., dual-degree), the duration might be longer.  2. **Work Hours Limit:**    - You are generally allowed to work full-time (up to 40 hours per week) while on this visa, but you can also choose to work part-time.    - There is no specific limit on the number of hours you can work in a week, as long as it does not exceed full-time.  ### Other Possible Visa Types If your situation differs or if you have any other type of visa, here are some additional points:  1. **Graduate Work Stream (GWS) Visa:**    - If you were granted the GWS visa, which is part of the Skilled Occupation List (SOL), you can stay for up to 3 years.    - The work hours limit is similar to the PSW; you are allowed to work full-time or part-time.  2. **Temporary Graduate Visa:**    - This visa allows you to stay in Australia for up to 18 months after completing your studies.    - You can work full-time during this period, but there might be restrictions if you want to extend the visa beyond its initial term.  ### Important Considerations - **Eligibility:** Ensure that you meet all eligibility criteria for the PSW or any other visa type. This includes having a valid offer of employment in certain cases. - **Visa Conditions:** Always check your specific visa conditions, as they can vary based on individual circumstances and the type of visa granted.  ### Next Steps 1. **Review Your Visa Information:** Log into the Department of Home Affairs website or use their mobile app to review your visa details. 2. **Seek Professional Advice:** If you are unsure about any aspect of your visa, consider consulting with a registered migration agent or an immigration lawyer for personalized advice.  If you have specific questions about your situation, it's best to contact the Department of Home Affairs directly or seek professional assistance.</t>
+          <t>Congratulations on graduating! The specifics of your post-study work visa (also known as the Graduate Work Stream of the Temporary Graduate Visa) depend on several factors, including the type of visa you have been granted. Here’s a general overview:  ### Duration of Stay: - **Temporary Graduate Visa (485):** If you are eligible for this visa, it typically allows you to stay in Australia for up to 18 months after your course completion.    - **Post-Study Work Visa (Subclass 790 or Subclass 791):** This is a more recent visa that replaced the Temporary Graduate Visa. It also allows you to work and live in Australia for up to 3 years, depending on the length of your studies.  ### Work Hours Limit: - **Temporary Graduate Visa (485):** You are generally allowed to work full-time or part-time while holding this visa.    - **Post-Study Work Visa (Subclass 790/791):** Similar to the Temporary Graduate Visa, you can also work full-time or part-time.  ### Additional Considerations: - **Eligibility:** Ensure that you meet all eligibility criteria for the post-study work visa. This includes having completed a qualifying course and meeting English language requirements.    - **Visa Conditions:** Always check the specific conditions of your visa, as there may be additional restrictions or obligations.  For precise details about your visa, including any specific conditions or limitations, you should refer to the official Australian Government Department of Home Affairs website or consult with an immigration advisor. They can provide tailored advice based on your individual circumstances.</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>You can stay in Australia under the Post-Higher Education Work stream of the Subclass 485 Temporary Graduate visa for usually between 2 and 3 years, depending on your qualification. There is no stated fortnightly work-hour cap; you can work in Australia without this restriction according to the information provided. Always check the visa grant notice/VEVO for specific conditions attached to your individual grant.</t>
+          <t>You can stay in Australia for usually between 2 and 3 years under the Post-Higher Education Work stream of the subclass 485 Temporary Graduate visa. There is no stated work-hour restriction for this stream. Source: [Subclass 485 — Temporary Graduate visa].</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>subclass_500_student.txt (0.807); subclass_485_temporary_graduate.txt (0.761); subclass_485_temporary_graduate.txt (0.759)</t>
+          <t>subclass_500_student.txt (0.78); subclass_485_temporary_graduate.txt (0.754); subclass_485_temporary_graduate.txt (0.742)</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr"/>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>I'm sorry, but I don't have access to your specific circumstances or the details of your Subclass 482 visa application. The approval of a Subclass 482 visa depends on several factors and is determined by the Australian Government based on the information provided in your application.  To increase your chances of approval, make sure you:  1. Meet all eligibility criteria: This includes having a valid job offer from an eligible employer, meeting skill level requirements, and ensuring that there are no suitable Australian workers available for the position. 2. Provide comprehensive documentation: Ensure that all required documents are accurate, up-to-date, and submitted on time. 3. Address any potential issues: If you have any gaps in your employment history or other concerns, address them proactively by providing supporting evidence.  If you're unsure about your application's status or need guidance, consider consulting with a registered migration agent who can provide personalized advice based on your specific situation.</t>
+          <t>I'm sorry, but I don't have access to your specific circumstances or the details of your application. The approval of a Subclass 482 visa depends on various factors and is determined by the Australian Government's Department of Home Affairs.  To increase your chances of approval, you should ensure that:  1. You meet all eligibility criteria for the Subclass 482 visa. 2. Your nomination or occupation is on the relevant list (e.g., Skilled Occupation List - SOL). 3. You have a valid job offer from an Australian employer who has met certain requirements. 4. Your skills and experience match the requirements of your nominated position. 5. You meet the health, character, and other conditions required for the visa.  If you're unsure about any aspect of your application or need guidance on how to improve it, I recommend consulting with a registered migration agent or solicitor who specializes in Australian immigration law. They can provide personalized advice based on your specific situation.</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>subclass_482_skills_in_demand.txt (0.743); subclass_482_skills_in_demand.txt (0.69); subclass_485_temporary_graduate.txt (0.685)</t>
+          <t>subclass_482_skills_in_demand.txt (0.754); subclass_482_skills_in_demand.txt (0.744); subclass_482_skills_in_demand.txt (0.726)</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Whether to accept a job that pays slightly below the Specialist Skills Income Threshold depends on several factors:  1. **Job Satisfaction**: Consider whether the role aligns with your career goals and interests. A job you enjoy can be more fulfilling than one that just meets financial expectations.  2. **Future Prospects**: Check if there are opportunities for advancement or salary increases within the organization. Sometimes, starting at a lower level can lead to better long-term prospects.  3. **Benefits Package**: Look beyond just the salary. Consider other benefits such as health insurance, retirement plans, vacation time, and professional development opportunities.  4. **Market Conditions**: Research the local job market and industry standards. If your skills are in high demand, you might find that the pay will increase over time or that similar roles command higher salaries.  5. **Personal Financial Situation**: Assess your current financial needs and whether this salary is sufficient to cover your living expenses and any other commitments.  6. **Negotiation**: Sometimes, it's worth negotiating for a higher starting salary or better terms. You might be able to secure a raise in the future based on performance reviews or company policies.  7. **Alternative Opportunities**: Consider if there are other positions available that meet both your skill level and desired income. It’s often beneficial to have multiple options before making a decision.  8. **Consultation**: If you're unsure, it might be helpful to consult with a career advisor or mentor who can provide personalized advice based on your specific situation.  Ultimately, the decision should balance your immediate financial needs with long-term professional growth and satisfaction.</t>
+          <t>Whether to accept a job that pays slightly below the Specialist Skills Income Threshold depends on several factors:  1. **Job Satisfaction**: Consider whether the role aligns with your career goals and interests. A job you enjoy can be more fulfilling than one that just meets financial expectations.  2. **Future Prospects**: Check if there are opportunities for advancement or salary increases within the organization. Sometimes, starting at a lower level can lead to better long-term prospects.  3. **Benefits Package**: Look beyond just the salary. Consider other benefits such as health insurance, retirement plans, vacation time, and professional development opportunities.  4. **Market Conditions**: Research the current job market in your field. If salaries are generally low or stagnant, it might be more challenging to find a higher-paying position later on.  5. **Personal Financial Situation**: Assess whether the salary is sufficient for your needs. Consider living expenses, debt obligations, and savings goals.  6. **Negotiation**: Sometimes you can negotiate better terms, such as a higher starting salary, additional vacation days, or other perks.  7. **Alternative Opportunities**: Explore if there are other positions available that might offer a more competitive salary while still aligning with your career aspirations.  If the job offers significant benefits and aligns well with your long-term goals, it could be worth considering even if the pay is slightly below the threshold. However, if you feel the financial strain will significantly impact your quality of life or professional growth, it might be better to look for a position that meets or exceeds the Specialist Skills Income Threshold.</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>subclass_482_skills_in_demand.txt (0.666); subclass_482_skills_in_demand.txt (0.616); subclass_482_skills_in_demand.txt (0.593)</t>
+          <t>subclass_482_skills_in_demand.txt (0.659); subclass_482_skills_in_demand.txt (0.62); subclass_482_skills_in_demand.txt (0.62)</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>whm_6_month_work_limitation.txt (0.542); subclass_417_working_holiday.txt (0.492); subclass_417_working_holiday.txt (0.487)</t>
+          <t>whm_6_month_work_limitation.txt (0.517); subclass_417_working_holiday.txt (0.509); subclass_417_working_holiday.txt (0.508)</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
@@ -1525,17 +1525,17 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>In Australia, if you're on a Working Holiday Visa (subclass 417 or 462), there are specific rules regarding how long you can work and change employers. Generally, your visa allows you to work for up to 8 consecutive months with the same employer before you must leave the country or apply for another visa.  However, after those 8 months, you have a few options:  1. **Leave Australia**: You need to exit the country within 30 days of exceeding the 8-month limit. 2. **Apply for a New Visa**: If you want to continue working on the same farm, you can apply for a new visa that allows you to stay and work longer. This might include applying for a Temporary Skill Shortage (TSS) visa or another appropriate visa category.  It's important to note that: - You cannot simply keep working without changing your visa status. - The process of applying for a new visa should be done well in advance, as it can take some time and there are specific requirements you need to meet.  Always check the latest information from the Australian Government’s Department of Home Affairs website or consult with an immigration advisor to ensure you follow all necessary steps correctly.</t>
+          <t>In Australia, if you're on a Working Holiday Visa (subclass 417 or 462), there are specific rules regarding how long you can work and change employers. After 8 months of continuous employment with one employer, you generally need to leave the job for at least 30 days before returning to that same employer.  However, if you're still within your visa validity period (12 or 36 months), you may be able to return to the same farm after this 30-day break. It's important to note that:  1. **Check Your Visa Conditions:** Always refer to the specific conditions of your Working Holiday Visa. The Australian Government’s Department of Home Affairs website is a reliable source for detailed information.  2. **Employer Approval:** Some employers may have internal policies requiring them to approve you returning after the 30-day break, so it's best to check with your employer.  3. **Documentation:** Keep all relevant documentation and records related to your employment history, as this can be useful if there are any queries about your visa compliance.  4. **Consultation:** If you're unsure or need further clarification, consulting the Department of Home Affairs directly or seeking advice from a registered migration agent could provide peace of mind.  Always ensure that you comply with Australian immigration laws to avoid potential issues with your visa status.</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Based on the information provided, you are not required to seek permission to continue working for the same farm beyond 6 months if your work falls under the exemption for plant and animal cultivation anywhere in Australia. Since fruit picking is a form of plant cultivation, this activity qualifies under the specified exemptions.  Therefore, you do not need permission to keep working for the same farm after 8 months, as long as the work continues to be within the scope of plant cultivation. This is detailed in the exemptions section from 1 January 2024, which states that "plant and animal cultivation anywhere in Australia" is an exemption to the 6-month work limitation.  Reference: [Source: whm_6_month_work_limitation.txt]</t>
+          <t>I don't have enough information in my sources to answer that. However, based on the context provided, your work as fruit picking would typically fall under agricultural work. The exemptions list includes "plant and animal cultivation anywhere in Australia," which could potentially apply to your situation.  Given this, you might not need permission if your work continues to be within the scope of plant cultivation. Nonetheless, it's important to check the specific details or consult with the Department of Home Affairs directly for a definitive answer, as there may be additional criteria or changes since 1 January 2024 that could affect your situation.  For precise advice, please contact a registered migration agent or the Department of Home Affairs directly.</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>whm_6_month_work_limitation.txt (0.764); whm_6_month_work_limitation.txt (0.743); whm_6_month_work_limitation.txt (0.742)</t>
+          <t>whm_6_month_work_limitation.txt (0.739); whm_6_month_work_limitation.txt (0.724); whm_6_month_work_limitation.txt (0.718)</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>

</xml_diff>